<commit_message>
Update leaderboard with official teams and tie-ranking support
</commit_message>
<xml_diff>
--- a/leaderboard.xlsx
+++ b/leaderboard.xlsx
@@ -397,99 +397,165 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:C14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Rank</v>
+      </c>
+      <c r="B1" t="str">
         <v>Team Name</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Points</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>ByteBandits</v>
-      </c>
-      <c r="B2">
-        <v>1450</v>
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Hash-Cracks</v>
+      </c>
+      <c r="C2">
+        <v>1100</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>NullPointers</v>
-      </c>
-      <c r="B3">
-        <v>1320</v>
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>F Society</v>
+      </c>
+      <c r="C3">
+        <v>950</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>CyberKnights</v>
-      </c>
-      <c r="B4">
-        <v>1150</v>
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Elite Minds</v>
+      </c>
+      <c r="C4">
+        <v>900</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>0xBitShift</v>
-      </c>
-      <c r="B5">
-        <v>980</v>
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Black Hat</v>
+      </c>
+      <c r="C5">
+        <v>750</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>ShadowProtocol</v>
-      </c>
-      <c r="B6">
-        <v>870</v>
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Karunya</v>
+      </c>
+      <c r="C6">
+        <v>550</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>KernelPanic</v>
-      </c>
-      <c r="B7">
-        <v>750</v>
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="str">
+        <v>GriftiT</v>
+      </c>
+      <c r="C7">
+        <v>550</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
-        <v>BinaryBeasts</v>
-      </c>
-      <c r="B8">
-        <v>620</v>
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Space</v>
+      </c>
+      <c r="C8">
+        <v>500</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <v>PhishBusters</v>
-      </c>
-      <c r="B9">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Ctrl-Z</v>
+      </c>
+      <c r="C9">
         <v>500</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v>SYN_ACK_Attack</v>
-      </c>
-      <c r="B10">
-        <v>420</v>
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Data Dynamics</v>
+      </c>
+      <c r="C10">
+        <v>500</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v>CipherSquad</v>
-      </c>
-      <c r="B11">
-        <v>350</v>
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Vikings</v>
+      </c>
+      <c r="C11">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Mogers</v>
+      </c>
+      <c r="C12">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Data Dynamic</v>
+      </c>
+      <c r="C13">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Raiders</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>